<commit_message>
Add Smart Folder Import v1.7.2
</commit_message>
<xml_diff>
--- a/projects/RNA_Aptamer_Test/Experiments/Experiment_001/Results/DPV/peak_values.xlsx
+++ b/projects/RNA_Aptamer_Test/Experiments/Experiment_001/Results/DPV/peak_values.xlsx
@@ -503,19 +503,19 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="F2" t="n">
-        <v>13.074998</v>
+        <v>4.295834599999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="H2" t="n">
-        <v>13.074998</v>
+        <v>6.420831</v>
       </c>
       <c r="I2" t="n">
-        <v>9.829164999999996</v>
+        <v>2.124996400000001</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>

</xml_diff>